<commit_message>
Refine parsers and re-import all 8 pages with better card extraction
- cards.js: Rewrite parser to group flat sibling elements (img, h3, p, a)
  into card rows by scanning forward/backward from each h3
- carousel.js: Deduplicate CTAs by href, smarter slide dedup
- hero.js: Better background image detection, video support, CTA dedup
- hp-card-consolidator.js: New transformer to wrap sibling card items
- All 4 import scripts: Add card sibling consolidation before parsing
  (moves orphaned img/h3/p/a siblings into matched container)
- Re-imported all 8 pages: cards blocks now contain 3-6 items each
  instead of just the heading row

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tools/importer/reports/import-category-landing.report.xlsx
+++ b/tools/importer/reports/import-category-landing.report.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="56" uniqueCount="48">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="72" uniqueCount="58">
   <si>
     <t>_reportFile</t>
   </si>
@@ -52,7 +52,7 @@
     <t>category-landing</t>
   </si>
   <si>
-    <t>2026-04-08T08:59:57.440Z</t>
+    <t>2026-04-08T12:08:18.633Z</t>
   </si>
   <si>
     <t>desktops | HP® Official Site</t>
@@ -73,7 +73,7 @@
     <t>homepage</t>
   </si>
   <si>
-    <t>2026-04-08T00:33:46.325Z</t>
+    <t>2026-04-08T12:07:29.131Z</t>
   </si>
   <si>
     <t>Laptop Computers, Desktops, Printers, Ink &amp; Toner | HP® Official Site</t>
@@ -91,7 +91,7 @@
     <t>us-en/laptops-and-2-in-1s</t>
   </si>
   <si>
-    <t>2026-04-08T07:43:30.409Z</t>
+    <t>2026-04-08T12:08:08.991Z</t>
   </si>
   <si>
     <t>HP Laptop Computers and 2-in-1 PCs | HP® Official Site</t>
@@ -106,7 +106,7 @@
     <t>us-en/printers</t>
   </si>
   <si>
-    <t>2026-04-08T09:00:07.958Z</t>
+    <t>2026-04-08T12:08:28.718Z</t>
   </si>
   <si>
     <t>printers | HP® Official Site</t>
@@ -127,7 +127,7 @@
     <t>content-editorial</t>
   </si>
   <si>
-    <t>2026-04-08T07:46:18.216Z</t>
+    <t>2026-04-08T12:06:12.929Z</t>
   </si>
   <si>
     <t>Sustainable Impact | HP® Official Site</t>
@@ -136,6 +136,24 @@
     <t>https://www.hp.com/us-en/sustainable-impact.html</t>
   </si>
   <si>
+    <t>us-en/all-in-plan/printers.report.json</t>
+  </si>
+  <si>
+    <t>us-en/all-in-plan/printers</t>
+  </si>
+  <si>
+    <t>product-marketing</t>
+  </si>
+  <si>
+    <t>2026-04-08T12:06:08.312Z</t>
+  </si>
+  <si>
+    <t>HP All-In Plan – Printer Plans | HP® Official Site</t>
+  </si>
+  <si>
+    <t>https://www.hp.com/us-en/all-in-plan/printers.html</t>
+  </si>
+  <si>
     <t>us-en/printers/smart-tank.report.json</t>
   </si>
   <si>
@@ -145,16 +163,28 @@
     <t>us-en/printers/smart-tank</t>
   </si>
   <si>
-    <t>product-marketing</t>
-  </si>
-  <si>
-    <t>2026-04-08T07:43:45.730Z</t>
+    <t>2026-04-08T12:05:43.806Z</t>
   </si>
   <si>
     <t>HP Smart Tank Printers – Refillable Ink Tank Printers | HP® Official Site</t>
   </si>
   <si>
     <t>https://www.hp.com/us-en/printers/smart-tank.html</t>
+  </si>
+  <si>
+    <t>us-en/software/microsoft-copilot-pcs-for-home.report.json</t>
+  </si>
+  <si>
+    <t>us-en/software/microsoft-copilot-pcs-for-home</t>
+  </si>
+  <si>
+    <t>2026-04-08T12:05:55.964Z</t>
+  </si>
+  <si>
+    <t>Microsoft Copilot+ PCs For Home | HP® Official Site</t>
+  </si>
+  <si>
+    <t>https://www.hp.com/us-en/software/microsoft-copilot-pcs-for-home.html</t>
   </si>
 </sst>
 </file>
@@ -543,12 +573,11 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:H7"/>
+  <dimension ref="A1:H9"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
-    <col min="1" max="1" width="39" customWidth="1"/>
-    <col min="2" max="2" width="50" customWidth="1"/>
-    <col min="3" max="3" width="27" customWidth="1"/>
+    <col min="1" max="2" width="50" customWidth="1"/>
+    <col min="3" max="3" width="47" customWidth="1"/>
     <col min="5" max="5" width="19" customWidth="1"/>
     <col min="6" max="6" width="26" customWidth="1"/>
     <col min="7" max="8" width="50" customWidth="1"/>
@@ -715,25 +744,77 @@
         <v>41</v>
       </c>
       <c r="B7" t="s">
+        <v>9</v>
+      </c>
+      <c r="C7" t="s">
         <v>42</v>
-      </c>
-      <c r="C7" t="s">
-        <v>43</v>
       </c>
       <c r="D7" t="s">
         <v>11</v>
       </c>
       <c r="E7" t="s">
+        <v>43</v>
+      </c>
+      <c r="F7" t="s">
         <v>44</v>
       </c>
-      <c r="F7" t="s">
+      <c r="G7" t="s">
         <v>45</v>
       </c>
-      <c r="G7" t="s">
+      <c r="H7" t="s">
         <v>46</v>
       </c>
-      <c r="H7" t="s">
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
         <v>47</v>
+      </c>
+      <c r="B8" t="s">
+        <v>48</v>
+      </c>
+      <c r="C8" t="s">
+        <v>49</v>
+      </c>
+      <c r="D8" t="s">
+        <v>11</v>
+      </c>
+      <c r="E8" t="s">
+        <v>43</v>
+      </c>
+      <c r="F8" t="s">
+        <v>50</v>
+      </c>
+      <c r="G8" t="s">
+        <v>51</v>
+      </c>
+      <c r="H8" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>53</v>
+      </c>
+      <c r="B9" t="s">
+        <v>9</v>
+      </c>
+      <c r="C9" t="s">
+        <v>54</v>
+      </c>
+      <c r="D9" t="s">
+        <v>11</v>
+      </c>
+      <c r="E9" t="s">
+        <v>43</v>
+      </c>
+      <c r="F9" t="s">
+        <v>55</v>
+      </c>
+      <c r="G9" t="s">
+        <v>56</v>
+      </c>
+      <c r="H9" t="s">
+        <v>57</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Improve content quality and add Tier 2 pages
Content quality:
- New parsers: icon-grid, product-card, comparison-table, feature-carousel
- Homepage import script uses icon-grid for Our Products, product-card for Must Haves
- hp-cleanup transformer removes skip links, Related links, carousel placeholder
  text, and modal elements
- Re-imported all 8 Tier 1 pages with cleaner output

Tier 2 pages (5 new):
- HP Information (/us-en/hp-information)
- Newsroom (/us-en/newsroom)
- Monitors (/us-en/monitors)
- Accessories (/us-en/accessories)
- Business Solutions (/us-en/business-solutions)

Total: 13 HP pages imported across 4 templates

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tools/importer/reports/import-category-landing.report.xlsx
+++ b/tools/importer/reports/import-category-landing.report.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="72" uniqueCount="58">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="112" uniqueCount="84">
   <si>
     <t>_reportFile</t>
   </si>
@@ -37,22 +37,52 @@
     <t>url</t>
   </si>
   <si>
+    <t>us-en/accessories.report.json</t>
+  </si>
+  <si>
+    <t>[]</t>
+  </si>
+  <si>
+    <t>us-en/accessories</t>
+  </si>
+  <si>
+    <t>success</t>
+  </si>
+  <si>
+    <t>category-landing</t>
+  </si>
+  <si>
+    <t>2026-04-08T12:29:42.343Z</t>
+  </si>
+  <si>
+    <t>404 | HP® Official Site</t>
+  </si>
+  <si>
+    <t>https://www.hp.com/us-en/accessories.html</t>
+  </si>
+  <si>
+    <t>us-en/business-solutions.report.json</t>
+  </si>
+  <si>
+    <t>us-en/business-solutions</t>
+  </si>
+  <si>
+    <t>2026-04-08T12:29:55.182Z</t>
+  </si>
+  <si>
+    <t>business-solutions | HP® Official Site</t>
+  </si>
+  <si>
+    <t>https://www.hp.com/us-en/business-solutions.html</t>
+  </si>
+  <si>
     <t>us-en/desktops.report.json</t>
   </si>
   <si>
-    <t>[]</t>
-  </si>
-  <si>
     <t>us-en/desktops</t>
   </si>
   <si>
-    <t>success</t>
-  </si>
-  <si>
-    <t>category-landing</t>
-  </si>
-  <si>
-    <t>2026-04-08T12:08:18.633Z</t>
+    <t>2026-04-08T12:27:04.469Z</t>
   </si>
   <si>
     <t>desktops | HP® Official Site</t>
@@ -64,7 +94,7 @@
     <t>us-en/home.report.json</t>
   </si>
   <si>
-    <t>["carousel","cards","cards","cards","cards","cards","hero","hero","hero","hero","columns"]</t>
+    <t>["carousel","icon-grid","product-card","cards","cards","cards","hero","hero","hero","hero","columns"]</t>
   </si>
   <si>
     <t>us-en/home</t>
@@ -73,7 +103,7 @@
     <t>homepage</t>
   </si>
   <si>
-    <t>2026-04-08T12:07:29.131Z</t>
+    <t>2026-04-08T12:26:47.046Z</t>
   </si>
   <si>
     <t>Laptop Computers, Desktops, Printers, Ink &amp; Toner | HP® Official Site</t>
@@ -82,6 +112,27 @@
     <t>https://www.hp.com/us-en/home.html</t>
   </si>
   <si>
+    <t>us-en/hp-information.report.json</t>
+  </si>
+  <si>
+    <t>["cards","cards","cards"]</t>
+  </si>
+  <si>
+    <t>us-en/hp-information</t>
+  </si>
+  <si>
+    <t>content-editorial</t>
+  </si>
+  <si>
+    <t>2026-04-08T12:29:21.774Z</t>
+  </si>
+  <si>
+    <t>About Us | HP® Official Site</t>
+  </si>
+  <si>
+    <t>https://www.hp.com/us-en/hp-information.html</t>
+  </si>
+  <si>
     <t>us-en/laptops-and-2-in-1s.report.json</t>
   </si>
   <si>
@@ -91,7 +142,7 @@
     <t>us-en/laptops-and-2-in-1s</t>
   </si>
   <si>
-    <t>2026-04-08T12:08:08.991Z</t>
+    <t>2026-04-08T12:26:54.692Z</t>
   </si>
   <si>
     <t>HP Laptop Computers and 2-in-1 PCs | HP® Official Site</t>
@@ -100,13 +151,43 @@
     <t>https://www.hp.com/us-en/laptops-and-2-in-1s.html</t>
   </si>
   <si>
+    <t>us-en/monitors.report.json</t>
+  </si>
+  <si>
+    <t>us-en/monitors</t>
+  </si>
+  <si>
+    <t>2026-04-08T12:29:36.760Z</t>
+  </si>
+  <si>
+    <t>https://www.hp.com/us-en/monitors.html</t>
+  </si>
+  <si>
+    <t>us-en/newsroom.report.json</t>
+  </si>
+  <si>
+    <t>["hero"]</t>
+  </si>
+  <si>
+    <t>us-en/newsroom</t>
+  </si>
+  <si>
+    <t>2026-04-08T12:29:32.977Z</t>
+  </si>
+  <si>
+    <t>Newsroom | HP® Official Site</t>
+  </si>
+  <si>
+    <t>https://www.hp.com/us-en/newsroom.html</t>
+  </si>
+  <si>
     <t>us-en/printers.report.json</t>
   </si>
   <si>
     <t>us-en/printers</t>
   </si>
   <si>
-    <t>2026-04-08T12:08:28.718Z</t>
+    <t>2026-04-08T12:27:15.644Z</t>
   </si>
   <si>
     <t>printers | HP® Official Site</t>
@@ -124,10 +205,7 @@
     <t>us-en/sustainable-impact</t>
   </si>
   <si>
-    <t>content-editorial</t>
-  </si>
-  <si>
-    <t>2026-04-08T12:06:12.929Z</t>
+    <t>2026-04-08T12:27:53.823Z</t>
   </si>
   <si>
     <t>Sustainable Impact | HP® Official Site</t>
@@ -145,7 +223,7 @@
     <t>product-marketing</t>
   </si>
   <si>
-    <t>2026-04-08T12:06:08.312Z</t>
+    <t>2026-04-08T12:27:49.476Z</t>
   </si>
   <si>
     <t>HP All-In Plan – Printer Plans | HP® Official Site</t>
@@ -163,7 +241,7 @@
     <t>us-en/printers/smart-tank</t>
   </si>
   <si>
-    <t>2026-04-08T12:05:43.806Z</t>
+    <t>2026-04-08T12:27:21.397Z</t>
   </si>
   <si>
     <t>HP Smart Tank Printers – Refillable Ink Tank Printers | HP® Official Site</t>
@@ -178,7 +256,7 @@
     <t>us-en/software/microsoft-copilot-pcs-for-home</t>
   </si>
   <si>
-    <t>2026-04-08T12:05:55.964Z</t>
+    <t>2026-04-08T12:27:35.692Z</t>
   </si>
   <si>
     <t>Microsoft Copilot+ PCs For Home | HP® Official Site</t>
@@ -573,7 +651,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:H9"/>
+  <dimension ref="A1:H14"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="2" width="50" customWidth="1"/>
@@ -640,36 +718,36 @@
         <v>16</v>
       </c>
       <c r="B3" t="s">
+        <v>9</v>
+      </c>
+      <c r="C3" t="s">
         <v>17</v>
       </c>
-      <c r="C3" t="s">
+      <c r="D3" t="s">
+        <v>11</v>
+      </c>
+      <c r="E3" t="s">
+        <v>12</v>
+      </c>
+      <c r="F3" t="s">
         <v>18</v>
       </c>
-      <c r="D3" t="s">
-        <v>11</v>
-      </c>
-      <c r="E3" t="s">
+      <c r="G3" t="s">
         <v>19</v>
       </c>
-      <c r="F3" t="s">
+      <c r="H3" t="s">
         <v>20</v>
-      </c>
-      <c r="G3" t="s">
-        <v>21</v>
-      </c>
-      <c r="H3" t="s">
-        <v>22</v>
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="B4" t="s">
-        <v>24</v>
+        <v>9</v>
       </c>
       <c r="C4" t="s">
-        <v>25</v>
+        <v>22</v>
       </c>
       <c r="D4" t="s">
         <v>11</v>
@@ -678,73 +756,73 @@
         <v>12</v>
       </c>
       <c r="F4" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="G4" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="H4" t="s">
-        <v>28</v>
+        <v>25</v>
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
+        <v>26</v>
+      </c>
+      <c r="B5" t="s">
+        <v>27</v>
+      </c>
+      <c r="C5" t="s">
+        <v>28</v>
+      </c>
+      <c r="D5" t="s">
+        <v>11</v>
+      </c>
+      <c r="E5" t="s">
         <v>29</v>
       </c>
-      <c r="B5" t="s">
-        <v>9</v>
-      </c>
-      <c r="C5" t="s">
+      <c r="F5" t="s">
         <v>30</v>
       </c>
-      <c r="D5" t="s">
-        <v>11</v>
-      </c>
-      <c r="E5" t="s">
-        <v>12</v>
-      </c>
-      <c r="F5" t="s">
+      <c r="G5" t="s">
         <v>31</v>
       </c>
-      <c r="G5" t="s">
+      <c r="H5" t="s">
         <v>32</v>
-      </c>
-      <c r="H5" t="s">
-        <v>33</v>
       </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
+        <v>33</v>
+      </c>
+      <c r="B6" t="s">
         <v>34</v>
       </c>
-      <c r="B6" t="s">
+      <c r="C6" t="s">
         <v>35</v>
       </c>
-      <c r="C6" t="s">
+      <c r="D6" t="s">
+        <v>11</v>
+      </c>
+      <c r="E6" t="s">
         <v>36</v>
       </c>
-      <c r="D6" t="s">
-        <v>11</v>
-      </c>
-      <c r="E6" t="s">
+      <c r="F6" t="s">
         <v>37</v>
       </c>
-      <c r="F6" t="s">
+      <c r="G6" t="s">
         <v>38</v>
       </c>
-      <c r="G6" t="s">
+      <c r="H6" t="s">
         <v>39</v>
-      </c>
-      <c r="H6" t="s">
-        <v>40</v>
       </c>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
+        <v>40</v>
+      </c>
+      <c r="B7" t="s">
         <v>41</v>
-      </c>
-      <c r="B7" t="s">
-        <v>9</v>
       </c>
       <c r="C7" t="s">
         <v>42</v>
@@ -753,68 +831,198 @@
         <v>11</v>
       </c>
       <c r="E7" t="s">
+        <v>12</v>
+      </c>
+      <c r="F7" t="s">
         <v>43</v>
       </c>
-      <c r="F7" t="s">
+      <c r="G7" t="s">
         <v>44</v>
       </c>
-      <c r="G7" t="s">
+      <c r="H7" t="s">
         <v>45</v>
-      </c>
-      <c r="H7" t="s">
-        <v>46</v>
       </c>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
+        <v>46</v>
+      </c>
+      <c r="B8" t="s">
+        <v>9</v>
+      </c>
+      <c r="C8" t="s">
         <v>47</v>
       </c>
-      <c r="B8" t="s">
+      <c r="D8" t="s">
+        <v>11</v>
+      </c>
+      <c r="E8" t="s">
+        <v>12</v>
+      </c>
+      <c r="F8" t="s">
         <v>48</v>
       </c>
-      <c r="C8" t="s">
+      <c r="G8" t="s">
+        <v>14</v>
+      </c>
+      <c r="H8" t="s">
         <v>49</v>
-      </c>
-      <c r="D8" t="s">
-        <v>11</v>
-      </c>
-      <c r="E8" t="s">
-        <v>43</v>
-      </c>
-      <c r="F8" t="s">
-        <v>50</v>
-      </c>
-      <c r="G8" t="s">
-        <v>51</v>
-      </c>
-      <c r="H8" t="s">
-        <v>52</v>
       </c>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
+        <v>50</v>
+      </c>
+      <c r="B9" t="s">
+        <v>51</v>
+      </c>
+      <c r="C9" t="s">
+        <v>52</v>
+      </c>
+      <c r="D9" t="s">
+        <v>11</v>
+      </c>
+      <c r="E9" t="s">
+        <v>36</v>
+      </c>
+      <c r="F9" t="s">
         <v>53</v>
       </c>
-      <c r="B9" t="s">
+      <c r="G9" t="s">
+        <v>54</v>
+      </c>
+      <c r="H9" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>56</v>
+      </c>
+      <c r="B10" t="s">
         <v>9</v>
       </c>
-      <c r="C9" t="s">
-        <v>54</v>
-      </c>
-      <c r="D9" t="s">
-        <v>11</v>
-      </c>
-      <c r="E9" t="s">
-        <v>43</v>
-      </c>
-      <c r="F9" t="s">
-        <v>55</v>
-      </c>
-      <c r="G9" t="s">
-        <v>56</v>
-      </c>
-      <c r="H9" t="s">
+      <c r="C10" t="s">
         <v>57</v>
+      </c>
+      <c r="D10" t="s">
+        <v>11</v>
+      </c>
+      <c r="E10" t="s">
+        <v>12</v>
+      </c>
+      <c r="F10" t="s">
+        <v>58</v>
+      </c>
+      <c r="G10" t="s">
+        <v>59</v>
+      </c>
+      <c r="H10" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>61</v>
+      </c>
+      <c r="B11" t="s">
+        <v>62</v>
+      </c>
+      <c r="C11" t="s">
+        <v>63</v>
+      </c>
+      <c r="D11" t="s">
+        <v>11</v>
+      </c>
+      <c r="E11" t="s">
+        <v>36</v>
+      </c>
+      <c r="F11" t="s">
+        <v>64</v>
+      </c>
+      <c r="G11" t="s">
+        <v>65</v>
+      </c>
+      <c r="H11" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>67</v>
+      </c>
+      <c r="B12" t="s">
+        <v>9</v>
+      </c>
+      <c r="C12" t="s">
+        <v>68</v>
+      </c>
+      <c r="D12" t="s">
+        <v>11</v>
+      </c>
+      <c r="E12" t="s">
+        <v>69</v>
+      </c>
+      <c r="F12" t="s">
+        <v>70</v>
+      </c>
+      <c r="G12" t="s">
+        <v>71</v>
+      </c>
+      <c r="H12" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>73</v>
+      </c>
+      <c r="B13" t="s">
+        <v>74</v>
+      </c>
+      <c r="C13" t="s">
+        <v>75</v>
+      </c>
+      <c r="D13" t="s">
+        <v>11</v>
+      </c>
+      <c r="E13" t="s">
+        <v>69</v>
+      </c>
+      <c r="F13" t="s">
+        <v>76</v>
+      </c>
+      <c r="G13" t="s">
+        <v>77</v>
+      </c>
+      <c r="H13" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="14" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>79</v>
+      </c>
+      <c r="B14" t="s">
+        <v>9</v>
+      </c>
+      <c r="C14" t="s">
+        <v>80</v>
+      </c>
+      <c r="D14" t="s">
+        <v>11</v>
+      </c>
+      <c r="E14" t="s">
+        <v>69</v>
+      </c>
+      <c r="F14" t="s">
+        <v>81</v>
+      </c>
+      <c r="G14" t="s">
+        <v>82</v>
+      </c>
+      <c r="H14" t="s">
+        <v>83</v>
       </c>
     </row>
   </sheetData>

</xml_diff>